<commit_message>
Latest bunch of updates
</commit_message>
<xml_diff>
--- a/assets/excel_example_data.xlsx
+++ b/assets/excel_example_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\he162696\REPOS\ExcelControlCharts\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8873ACB1-E16B-4936-80FD-D2A45FCF06A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8463144-33ED-475E-8594-6C617FF09DD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25080" yWindow="-60" windowWidth="25440" windowHeight="15270" tabRatio="752" activeTab="5" xr2:uid="{B4DE27E6-3CDA-4D86-9B4B-E26F47FA9977}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="752" firstSheet="5" activeTab="14" xr2:uid="{B4DE27E6-3CDA-4D86-9B4B-E26F47FA9977}"/>
   </bookViews>
   <sheets>
     <sheet name="Run charts" sheetId="14" r:id="rId1"/>
@@ -2015,7 +2015,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="698" row="1">
+  <wetp:taskpane dockstate="right" visibility="0" width="525" row="1">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -2034,12 +2034,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E91ED3F9-FD8B-42B8-9B02-B889A07F00F1}">
   <dimension ref="A1:B18"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.26953125" customWidth="1"/>
+    <col min="1" max="1" width="15.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -2047,7 +2047,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>40179</v>
       </c>
@@ -2055,7 +2055,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>40210</v>
       </c>
@@ -2063,7 +2063,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>40238</v>
       </c>
@@ -2071,7 +2071,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>40269</v>
       </c>
@@ -2079,7 +2079,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>40299</v>
       </c>
@@ -2087,7 +2087,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>40330</v>
       </c>
@@ -2095,7 +2095,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>40360</v>
       </c>
@@ -2103,7 +2103,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>40391</v>
       </c>
@@ -2111,7 +2111,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>40422</v>
       </c>
@@ -2119,7 +2119,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>40452</v>
       </c>
@@ -2127,7 +2127,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>40483</v>
       </c>
@@ -2135,7 +2135,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>40513</v>
       </c>
@@ -2143,7 +2143,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>40544</v>
       </c>
@@ -2151,7 +2151,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>40575</v>
       </c>
@@ -2159,7 +2159,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>40603</v>
       </c>
@@ -2167,7 +2167,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>40634</v>
       </c>
@@ -2175,7 +2175,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>40664</v>
       </c>
@@ -2195,12 +2195,12 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5A69703-9BBF-41C0-9DA0-7B57125EA047}">
   <dimension ref="A1:C37"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.54296875" customWidth="1"/>
+    <col min="1" max="1" width="25.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -2211,7 +2211,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>40725</v>
       </c>
@@ -2222,7 +2222,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>40756</v>
       </c>
@@ -2233,7 +2233,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>40787</v>
       </c>
@@ -2244,7 +2244,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>40817</v>
       </c>
@@ -2255,7 +2255,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>40848</v>
       </c>
@@ -2266,7 +2266,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>40878</v>
       </c>
@@ -2277,7 +2277,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>40909</v>
       </c>
@@ -2288,7 +2288,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>40940</v>
       </c>
@@ -2299,7 +2299,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>40969</v>
       </c>
@@ -2310,7 +2310,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>41000</v>
       </c>
@@ -2321,7 +2321,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>41030</v>
       </c>
@@ -2332,7 +2332,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>41061</v>
       </c>
@@ -2343,7 +2343,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>41091</v>
       </c>
@@ -2354,7 +2354,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>41122</v>
       </c>
@@ -2365,7 +2365,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>41153</v>
       </c>
@@ -2376,7 +2376,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>41183</v>
       </c>
@@ -2387,7 +2387,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>41214</v>
       </c>
@@ -2398,7 +2398,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>41244</v>
       </c>
@@ -2409,7 +2409,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>41275</v>
       </c>
@@ -2420,7 +2420,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>41306</v>
       </c>
@@ -2431,7 +2431,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>41334</v>
       </c>
@@ -2442,7 +2442,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>41365</v>
       </c>
@@ -2453,7 +2453,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>41395</v>
       </c>
@@ -2464,7 +2464,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>41426</v>
       </c>
@@ -2475,7 +2475,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>41456</v>
       </c>
@@ -2486,7 +2486,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>41487</v>
       </c>
@@ -2497,7 +2497,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>41518</v>
       </c>
@@ -2508,7 +2508,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>41548</v>
       </c>
@@ -2519,7 +2519,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>41579</v>
       </c>
@@ -2530,7 +2530,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <v>41609</v>
       </c>
@@ -2541,7 +2541,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>41640</v>
       </c>
@@ -2552,7 +2552,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>41671</v>
       </c>
@@ -2563,7 +2563,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>41699</v>
       </c>
@@ -2574,7 +2574,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>41730</v>
       </c>
@@ -2585,7 +2585,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <v>41760</v>
       </c>
@@ -2596,7 +2596,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>41791</v>
       </c>
@@ -2619,13 +2619,13 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1914B0D5-C1FB-4999-BF2C-D6B56FAF3D9A}">
   <dimension ref="A1:B68"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.7265625" customWidth="1"/>
-    <col min="2" max="2" width="11.7265625" customWidth="1"/>
+    <col min="1" max="1" width="16.7109375" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>13</v>
       </c>
@@ -2633,7 +2633,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>40761</v>
       </c>
@@ -2641,7 +2641,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>40781</v>
       </c>
@@ -2649,7 +2649,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>40786</v>
       </c>
@@ -2657,7 +2657,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>40799</v>
       </c>
@@ -2665,7 +2665,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>40800</v>
       </c>
@@ -2673,7 +2673,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>40826</v>
       </c>
@@ -2681,7 +2681,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>40872</v>
       </c>
@@ -2689,7 +2689,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>40884</v>
       </c>
@@ -2697,7 +2697,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>40896</v>
       </c>
@@ -2705,7 +2705,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>40901</v>
       </c>
@@ -2713,7 +2713,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>40920</v>
       </c>
@@ -2721,7 +2721,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>40924</v>
       </c>
@@ -2729,7 +2729,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>40927</v>
       </c>
@@ -2737,7 +2737,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>40942</v>
       </c>
@@ -2745,7 +2745,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>40956</v>
       </c>
@@ -2753,7 +2753,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>40965</v>
       </c>
@@ -2761,7 +2761,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>40973</v>
       </c>
@@ -2769,7 +2769,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>40988</v>
       </c>
@@ -2777,7 +2777,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>41009</v>
       </c>
@@ -2785,7 +2785,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>41015</v>
       </c>
@@ -2793,7 +2793,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>41018</v>
       </c>
@@ -2801,7 +2801,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>41019</v>
       </c>
@@ -2809,7 +2809,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>41075</v>
       </c>
@@ -2817,7 +2817,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>41192</v>
       </c>
@@ -2825,7 +2825,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>41193</v>
       </c>
@@ -2833,7 +2833,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>41226</v>
       </c>
@@ -2841,7 +2841,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>41235</v>
       </c>
@@ -2849,7 +2849,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>41244</v>
       </c>
@@ -2857,7 +2857,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>41263</v>
       </c>
@@ -2865,7 +2865,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <v>41275</v>
       </c>
@@ -2873,7 +2873,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>41276</v>
       </c>
@@ -2881,7 +2881,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>41292</v>
       </c>
@@ -2889,7 +2889,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>41305</v>
       </c>
@@ -2897,7 +2897,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>41323</v>
       </c>
@@ -2905,7 +2905,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <v>41324</v>
       </c>
@@ -2913,7 +2913,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>41359</v>
       </c>
@@ -2921,7 +2921,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
         <v>41375</v>
       </c>
@@ -2929,7 +2929,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
         <v>41380</v>
       </c>
@@ -2937,7 +2937,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
         <v>41401</v>
       </c>
@@ -2945,7 +2945,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
         <v>41439</v>
       </c>
@@ -2953,7 +2953,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
         <v>41442</v>
       </c>
@@ -2961,7 +2961,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
         <v>41467</v>
       </c>
@@ -2969,7 +2969,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
         <v>41470</v>
       </c>
@@ -2977,7 +2977,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
         <v>41481</v>
       </c>
@@ -2985,7 +2985,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
         <v>41494</v>
       </c>
@@ -2993,7 +2993,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
         <v>41514</v>
       </c>
@@ -3001,7 +3001,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
         <v>41523</v>
       </c>
@@ -3009,7 +3009,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
         <v>41526</v>
       </c>
@@ -3017,7 +3017,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
         <v>41534</v>
       </c>
@@ -3025,7 +3025,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
         <v>41555</v>
       </c>
@@ -3033,7 +3033,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
         <v>41579</v>
       </c>
@@ -3041,7 +3041,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
         <v>41617</v>
       </c>
@@ -3049,7 +3049,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
         <v>41625</v>
       </c>
@@ -3057,7 +3057,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
         <v>41638</v>
       </c>
@@ -3065,7 +3065,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
         <v>41647</v>
       </c>
@@ -3073,7 +3073,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
         <v>41648</v>
       </c>
@@ -3081,7 +3081,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
         <v>41678</v>
       </c>
@@ -3089,7 +3089,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
         <v>41701</v>
       </c>
@@ -3097,7 +3097,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
         <v>41704</v>
       </c>
@@ -3105,7 +3105,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
         <v>41711</v>
       </c>
@@ -3113,7 +3113,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
         <v>41733</v>
       </c>
@@ -3121,7 +3121,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
         <v>41752</v>
       </c>
@@ -3129,7 +3129,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
         <v>41763</v>
       </c>
@@ -3137,7 +3137,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
         <v>41794</v>
       </c>
@@ -3145,7 +3145,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
         <v>41800</v>
       </c>
@@ -3153,7 +3153,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
         <v>41801</v>
       </c>
@@ -3161,7 +3161,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
         <v>41802</v>
       </c>
@@ -3181,13 +3181,13 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94239D50-9E27-4C78-8D79-9458660D580C}">
   <dimension ref="A1:B68"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.7265625" customWidth="1"/>
-    <col min="2" max="2" width="14.26953125" customWidth="1"/>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="14.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>13</v>
       </c>
@@ -3195,7 +3195,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>40761</v>
       </c>
@@ -3203,7 +3203,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>40781</v>
       </c>
@@ -3211,7 +3211,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>40786</v>
       </c>
@@ -3219,7 +3219,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>40799</v>
       </c>
@@ -3227,7 +3227,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>40800</v>
       </c>
@@ -3235,7 +3235,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>40826</v>
       </c>
@@ -3243,7 +3243,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>40872</v>
       </c>
@@ -3251,7 +3251,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>40884</v>
       </c>
@@ -3259,7 +3259,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>40896</v>
       </c>
@@ -3267,7 +3267,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>40901</v>
       </c>
@@ -3275,7 +3275,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>40920</v>
       </c>
@@ -3283,7 +3283,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>40924</v>
       </c>
@@ -3291,7 +3291,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>40927</v>
       </c>
@@ -3299,7 +3299,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>40942</v>
       </c>
@@ -3307,7 +3307,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>40956</v>
       </c>
@@ -3315,7 +3315,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>40965</v>
       </c>
@@ -3323,7 +3323,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>40973</v>
       </c>
@@ -3331,7 +3331,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>40988</v>
       </c>
@@ -3339,7 +3339,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>41009</v>
       </c>
@@ -3347,7 +3347,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>41015</v>
       </c>
@@ -3355,7 +3355,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>41018</v>
       </c>
@@ -3363,7 +3363,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>41019</v>
       </c>
@@ -3371,7 +3371,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>41075</v>
       </c>
@@ -3379,7 +3379,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>41192</v>
       </c>
@@ -3387,7 +3387,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>41193</v>
       </c>
@@ -3395,7 +3395,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>41226</v>
       </c>
@@ -3403,7 +3403,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>41235</v>
       </c>
@@ -3411,7 +3411,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>41244</v>
       </c>
@@ -3419,7 +3419,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>41263</v>
       </c>
@@ -3427,7 +3427,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <v>41275</v>
       </c>
@@ -3435,7 +3435,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>41276</v>
       </c>
@@ -3443,7 +3443,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>41292</v>
       </c>
@@ -3451,7 +3451,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>41305</v>
       </c>
@@ -3459,7 +3459,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>41323</v>
       </c>
@@ -3467,7 +3467,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <v>41324</v>
       </c>
@@ -3475,7 +3475,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>41359</v>
       </c>
@@ -3483,7 +3483,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
         <v>41375</v>
       </c>
@@ -3491,7 +3491,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
         <v>41380</v>
       </c>
@@ -3499,7 +3499,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
         <v>41401</v>
       </c>
@@ -3507,7 +3507,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
         <v>41439</v>
       </c>
@@ -3515,7 +3515,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
         <v>41442</v>
       </c>
@@ -3523,7 +3523,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
         <v>41467</v>
       </c>
@@ -3531,7 +3531,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
         <v>41470</v>
       </c>
@@ -3539,7 +3539,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
         <v>41481</v>
       </c>
@@ -3547,7 +3547,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
         <v>41494</v>
       </c>
@@ -3555,7 +3555,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
         <v>41514</v>
       </c>
@@ -3563,7 +3563,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
         <v>41523</v>
       </c>
@@ -3571,7 +3571,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
         <v>41526</v>
       </c>
@@ -3579,7 +3579,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
         <v>41534</v>
       </c>
@@ -3587,7 +3587,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
         <v>41555</v>
       </c>
@@ -3595,7 +3595,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
         <v>41579</v>
       </c>
@@ -3603,7 +3603,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
         <v>41617</v>
       </c>
@@ -3611,7 +3611,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
         <v>41625</v>
       </c>
@@ -3619,7 +3619,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
         <v>41638</v>
       </c>
@@ -3627,7 +3627,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
         <v>41647</v>
       </c>
@@ -3635,7 +3635,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
         <v>41648</v>
       </c>
@@ -3643,7 +3643,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
         <v>41678</v>
       </c>
@@ -3651,7 +3651,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
         <v>41701</v>
       </c>
@@ -3659,7 +3659,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
         <v>41704</v>
       </c>
@@ -3667,7 +3667,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
         <v>41711</v>
       </c>
@@ -3675,7 +3675,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
         <v>41733</v>
       </c>
@@ -3683,7 +3683,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
         <v>41752</v>
       </c>
@@ -3691,7 +3691,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
         <v>41763</v>
       </c>
@@ -3699,7 +3699,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
         <v>41794</v>
       </c>
@@ -3707,7 +3707,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
         <v>41800</v>
       </c>
@@ -3715,7 +3715,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
         <v>41801</v>
       </c>
@@ -3723,7 +3723,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
         <v>41802</v>
       </c>
@@ -3743,14 +3743,14 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04EE4CED-F004-4308-9D32-54E31ABA6676}">
   <dimension ref="A1:C55"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.54296875" customWidth="1"/>
-    <col min="2" max="2" width="18.26953125" customWidth="1"/>
-    <col min="3" max="3" width="18.1796875" customWidth="1"/>
+    <col min="1" max="1" width="10.5703125" customWidth="1"/>
+    <col min="2" max="2" width="18.28515625" customWidth="1"/>
+    <col min="3" max="3" width="18.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>17</v>
       </c>
@@ -3761,7 +3761,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>30001</v>
       </c>
@@ -3772,7 +3772,7 @@
         <v>523.69630439918899</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>30002</v>
       </c>
@@ -3783,7 +3783,7 @@
         <v>612.97855293250404</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>30003</v>
       </c>
@@ -3794,7 +3794,7 @@
         <v>53.791361883082402</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>30006</v>
       </c>
@@ -3805,7 +3805,7 @@
         <v>763.71788755208001</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>30007</v>
       </c>
@@ -3816,7 +3816,7 @@
         <v>120.937392812274</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>30008</v>
       </c>
@@ -3827,7 +3827,7 @@
         <v>250.18601700482299</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>30009</v>
       </c>
@@ -3838,7 +3838,7 @@
         <v>155.492096238415</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>30010</v>
       </c>
@@ -3849,7 +3849,7 @@
         <v>484.71487638974497</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>30011</v>
       </c>
@@ -3860,7 +3860,7 @@
         <v>362.22213062348601</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>30012</v>
       </c>
@@ -3871,7 +3871,7 @@
         <v>188.92661245266899</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>30013</v>
       </c>
@@ -3882,7 +3882,7 @@
         <v>554.38476729293404</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>30014</v>
       </c>
@@ -3893,7 +3893,7 @@
         <v>616.73798367096595</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>30016</v>
       </c>
@@ -3904,7 +3904,7 @@
         <v>360.14733060718299</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>30017</v>
       </c>
@@ -3915,7 +3915,7 @@
         <v>245.612602349593</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>30018</v>
       </c>
@@ -3926,7 +3926,7 @@
         <v>263.56458385396098</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>30019</v>
       </c>
@@ -3937,7 +3937,7 @@
         <v>154.662422866464</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>30022</v>
       </c>
@@ -3948,7 +3948,7 @@
         <v>475.01588723983502</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>30023</v>
       </c>
@@ -3959,7 +3959,7 @@
         <v>38.933932087196098</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>30024</v>
       </c>
@@ -3970,7 +3970,7 @@
         <v>445.09655805302901</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>30025</v>
       </c>
@@ -3981,7 +3981,7 @@
         <v>28.797138877451101</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>30030</v>
       </c>
@@ -3992,7 +3992,7 @@
         <v>347.53640428645002</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>30033</v>
       </c>
@@ -4003,7 +4003,7 @@
         <v>7.56105136609865</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>30035</v>
       </c>
@@ -4014,7 +4014,7 @@
         <v>73.205601753135895</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>30036</v>
       </c>
@@ -4025,7 +4025,7 @@
         <v>118.113760661309</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>30037</v>
       </c>
@@ -4036,7 +4036,7 @@
         <v>273.33772770252301</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>30038</v>
       </c>
@@ -4047,7 +4047,7 @@
         <v>449.79320452069999</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>30043</v>
       </c>
@@ -4058,7 +4058,7 @@
         <v>172.37858327089199</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>30044</v>
       </c>
@@ -4069,7 +4069,7 @@
         <v>19.196258864521099</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>30055</v>
       </c>
@@ -4080,7 +4080,7 @@
         <v>321.858009678352</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30059</v>
       </c>
@@ -4091,7 +4091,7 @@
         <v>36.562995729262497</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>30060</v>
       </c>
@@ -4102,7 +4102,7 @@
         <v>19.964291547038801</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>30061</v>
       </c>
@@ -4113,7 +4113,7 @@
         <v>851.71637253913298</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>30062</v>
       </c>
@@ -4124,7 +4124,7 @@
         <v>198.94056071537</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>30064</v>
       </c>
@@ -4135,7 +4135,7 @@
         <v>302.39343012546601</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>30065</v>
       </c>
@@ -4146,7 +4146,7 @@
         <v>410.16347153987402</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>30067</v>
       </c>
@@ -4157,7 +4157,7 @@
         <v>45.865321481698501</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>30068</v>
       </c>
@@ -4168,7 +4168,7 @@
         <v>9.6673147877212795</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>30069</v>
       </c>
@@ -4179,7 +4179,7 @@
         <v>212.34495050224101</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>30073</v>
       </c>
@@ -4190,7 +4190,7 @@
         <v>38.922171910342897</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>30078</v>
       </c>
@@ -4201,7 +4201,7 @@
         <v>31.7378697563827</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>30080</v>
       </c>
@@ -4212,7 +4212,7 @@
         <v>285.63591146047099</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>30083</v>
       </c>
@@ -4223,7 +4223,7 @@
         <v>186.65606385109899</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>30084</v>
       </c>
@@ -4234,7 +4234,7 @@
         <v>33.981834097901299</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>30085</v>
       </c>
@@ -4245,7 +4245,7 @@
         <v>255.65466754394001</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>30086</v>
       </c>
@@ -4256,7 +4256,7 @@
         <v>242.02586647546701</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>30087</v>
       </c>
@@ -4267,7 +4267,7 @@
         <v>279.47621713842102</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>30088</v>
       </c>
@@ -4278,7 +4278,7 @@
         <v>619.26358555522597</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>30089</v>
       </c>
@@ -4289,7 +4289,7 @@
         <v>626.13019623701598</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>30092</v>
       </c>
@@ -4300,7 +4300,7 @@
         <v>145.67486270562799</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>30093</v>
       </c>
@@ -4311,7 +4311,7 @@
         <v>413.86209508712398</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>30094</v>
       </c>
@@ -4322,7 +4322,7 @@
         <v>111.262792653403</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>32000</v>
       </c>
@@ -4333,7 +4333,7 @@
         <v>685.58572378869201</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>32002</v>
       </c>
@@ -4344,7 +4344,7 @@
         <v>181.10791122010701</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>32003</v>
       </c>
@@ -4367,14 +4367,14 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58FCBDC3-2210-431B-920C-045503CD3E5D}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.54296875" customWidth="1"/>
-    <col min="2" max="2" width="17.453125" customWidth="1"/>
-    <col min="3" max="3" width="19.453125" customWidth="1"/>
+    <col min="1" max="1" width="10.5703125" customWidth="1"/>
+    <col min="2" max="2" width="17.42578125" customWidth="1"/>
+    <col min="3" max="3" width="19.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>17</v>
       </c>
@@ -4385,7 +4385,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -4396,7 +4396,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>10</v>
       </c>
@@ -4407,7 +4407,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
@@ -4418,7 +4418,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3</v>
       </c>
@@ -4429,7 +4429,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>4</v>
       </c>
@@ -4440,7 +4440,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>5</v>
       </c>
@@ -4451,7 +4451,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>6</v>
       </c>
@@ -4462,7 +4462,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>7</v>
       </c>
@@ -4473,7 +4473,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>8</v>
       </c>
@@ -4484,7 +4484,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>9</v>
       </c>
@@ -4507,14 +4507,14 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A214E1A-869F-4753-BE49-157F53D94478}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.54296875" customWidth="1"/>
-    <col min="2" max="2" width="17.453125" customWidth="1"/>
-    <col min="3" max="3" width="16.453125" customWidth="1"/>
+    <col min="1" max="1" width="10.5703125" customWidth="1"/>
+    <col min="2" max="2" width="17.42578125" customWidth="1"/>
+    <col min="3" max="3" width="16.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>17</v>
       </c>
@@ -4525,7 +4525,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -4536,7 +4536,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>10</v>
       </c>
@@ -4547,7 +4547,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
@@ -4558,7 +4558,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3</v>
       </c>
@@ -4569,7 +4569,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>4</v>
       </c>
@@ -4580,7 +4580,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>5</v>
       </c>
@@ -4591,7 +4591,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>6</v>
       </c>
@@ -4602,7 +4602,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>7</v>
       </c>
@@ -4613,7 +4613,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>8</v>
       </c>
@@ -4624,7 +4624,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>9</v>
       </c>
@@ -4647,13 +4647,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C5F4E47-B510-4624-9D60-F67EBAAAEFFA}">
   <dimension ref="A1:C22"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.26953125" customWidth="1"/>
-    <col min="2" max="2" width="9.26953125" customWidth="1"/>
+    <col min="1" max="1" width="21.28515625" customWidth="1"/>
+    <col min="2" max="2" width="9.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -4661,7 +4661,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>40179</v>
       </c>
@@ -4669,7 +4669,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>40210</v>
       </c>
@@ -4677,7 +4677,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>40238</v>
       </c>
@@ -4685,7 +4685,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>40269</v>
       </c>
@@ -4693,7 +4693,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>40299</v>
       </c>
@@ -4701,7 +4701,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>40330</v>
       </c>
@@ -4709,7 +4709,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>40360</v>
       </c>
@@ -4717,7 +4717,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>40391</v>
       </c>
@@ -4725,7 +4725,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>40422</v>
       </c>
@@ -4733,7 +4733,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>40452</v>
       </c>
@@ -4741,7 +4741,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>40483</v>
       </c>
@@ -4749,7 +4749,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>40513</v>
       </c>
@@ -4757,7 +4757,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>40544</v>
       </c>
@@ -4765,7 +4765,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>40575</v>
       </c>
@@ -4773,7 +4773,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>40603</v>
       </c>
@@ -4781,7 +4781,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>40634</v>
       </c>
@@ -4789,7 +4789,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>40664</v>
       </c>
@@ -4797,7 +4797,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C22" t="s">
         <v>3</v>
       </c>
@@ -4814,13 +4814,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6A1EBBE-BFA0-4C2A-8F00-D92C78290E2D}">
   <dimension ref="A1:C18"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="9.26953125" customWidth="1"/>
+    <col min="2" max="2" width="9.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -4831,7 +4831,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>40179</v>
       </c>
@@ -4842,7 +4842,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>40210</v>
       </c>
@@ -4853,7 +4853,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>40238</v>
       </c>
@@ -4864,7 +4864,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>40269</v>
       </c>
@@ -4875,7 +4875,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>40299</v>
       </c>
@@ -4886,7 +4886,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>40330</v>
       </c>
@@ -4897,7 +4897,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>40360</v>
       </c>
@@ -4908,7 +4908,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>40391</v>
       </c>
@@ -4919,7 +4919,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>40422</v>
       </c>
@@ -4930,7 +4930,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>40452</v>
       </c>
@@ -4941,7 +4941,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>40483</v>
       </c>
@@ -4952,7 +4952,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>40513</v>
       </c>
@@ -4963,7 +4963,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>40544</v>
       </c>
@@ -4974,7 +4974,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>40575</v>
       </c>
@@ -4985,7 +4985,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>40603</v>
       </c>
@@ -4996,7 +4996,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>40634</v>
       </c>
@@ -5007,7 +5007,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>40664</v>
       </c>
@@ -5030,14 +5030,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EECC891C-EE34-4005-8E2B-CDF24F154389}">
   <dimension ref="A1:C18"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" customWidth="1"/>
-    <col min="2" max="2" width="10.26953125" customWidth="1"/>
-    <col min="3" max="3" width="10.54296875" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" customWidth="1"/>
+    <col min="2" max="2" width="10.28515625" customWidth="1"/>
+    <col min="3" max="3" width="10.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -5048,7 +5048,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>40179</v>
       </c>
@@ -5059,7 +5059,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>40210</v>
       </c>
@@ -5070,7 +5070,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>40238</v>
       </c>
@@ -5081,7 +5081,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>40269</v>
       </c>
@@ -5092,7 +5092,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>40299</v>
       </c>
@@ -5103,7 +5103,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>40330</v>
       </c>
@@ -5114,7 +5114,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>40360</v>
       </c>
@@ -5125,7 +5125,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>40391</v>
       </c>
@@ -5136,7 +5136,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>40422</v>
       </c>
@@ -5147,7 +5147,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>40452</v>
       </c>
@@ -5158,7 +5158,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>40483</v>
       </c>
@@ -5169,7 +5169,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>40513</v>
       </c>
@@ -5180,7 +5180,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>40544</v>
       </c>
@@ -5191,7 +5191,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>40575</v>
       </c>
@@ -5202,7 +5202,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>40603</v>
       </c>
@@ -5213,7 +5213,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>40634</v>
       </c>
@@ -5224,7 +5224,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>40664</v>
       </c>
@@ -5247,13 +5247,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40DFCC3A-ECD0-4F8D-A9CF-8CB6D6A9105E}">
   <dimension ref="A1:C21"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="19.26953125" customWidth="1"/>
-    <col min="3" max="3" width="21.1796875" customWidth="1"/>
+    <col min="2" max="2" width="19.28515625" customWidth="1"/>
+    <col min="3" max="3" width="21.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -5264,7 +5264,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>36526</v>
       </c>
@@ -5275,7 +5275,7 @@
         <v>280443</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>36557</v>
       </c>
@@ -5286,7 +5286,7 @@
         <v>276823</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>36586</v>
       </c>
@@ -5297,7 +5297,7 @@
         <v>291681</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>36617</v>
       </c>
@@ -5308,7 +5308,7 @@
         <v>296155</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>36647</v>
       </c>
@@ -5319,7 +5319,7 @@
         <v>282343</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>36678</v>
       </c>
@@ -5330,7 +5330,7 @@
         <v>275888</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>36708</v>
       </c>
@@ -5341,7 +5341,7 @@
         <v>283867</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>36739</v>
       </c>
@@ -5352,7 +5352,7 @@
         <v>295251</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>36770</v>
       </c>
@@ -5363,7 +5363,7 @@
         <v>284468</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>36800</v>
       </c>
@@ -5374,7 +5374,7 @@
         <v>282529</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>36831</v>
       </c>
@@ -5385,7 +5385,7 @@
         <v>279618</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>36861</v>
       </c>
@@ -5396,7 +5396,7 @@
         <v>283932</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>36892</v>
       </c>
@@ -5407,7 +5407,7 @@
         <v>266629</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>36923</v>
       </c>
@@ -5418,7 +5418,7 @@
         <v>268091</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>36951</v>
       </c>
@@ -5429,7 +5429,7 @@
         <v>276803</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>36982</v>
       </c>
@@ -5440,7 +5440,7 @@
         <v>271578</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>37012</v>
       </c>
@@ -5451,7 +5451,7 @@
         <v>266005</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>37043</v>
       </c>
@@ -5462,7 +5462,7 @@
         <v>273520</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>37073</v>
       </c>
@@ -5473,7 +5473,7 @@
         <v>278574</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>37104</v>
       </c>
@@ -5496,13 +5496,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAC2F81D-A205-4DCE-B517-1B59A705DB10}">
   <dimension ref="A1:C18"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="17" customWidth="1"/>
-    <col min="3" max="3" width="14.453125" customWidth="1"/>
+    <col min="3" max="3" width="14.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -5513,7 +5513,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>40179</v>
       </c>
@@ -5524,7 +5524,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>40210</v>
       </c>
@@ -5535,7 +5535,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>40238</v>
       </c>
@@ -5546,7 +5546,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>40269</v>
       </c>
@@ -5557,7 +5557,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>40299</v>
       </c>
@@ -5568,7 +5568,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>40330</v>
       </c>
@@ -5579,7 +5579,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>40360</v>
       </c>
@@ -5590,7 +5590,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>40391</v>
       </c>
@@ -5601,7 +5601,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>40422</v>
       </c>
@@ -5612,7 +5612,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>40452</v>
       </c>
@@ -5623,7 +5623,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>40483</v>
       </c>
@@ -5634,7 +5634,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>40513</v>
       </c>
@@ -5645,7 +5645,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>40544</v>
       </c>
@@ -5656,7 +5656,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>40575</v>
       </c>
@@ -5667,7 +5667,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>40603</v>
       </c>
@@ -5678,7 +5678,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>40634</v>
       </c>
@@ -5689,7 +5689,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>40664</v>
       </c>
@@ -5712,13 +5712,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05B3C8B1-CD5A-4815-86FC-BCE94FBA487A}">
   <dimension ref="A1:C21"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="19.26953125" customWidth="1"/>
-    <col min="3" max="3" width="21.1796875" customWidth="1"/>
+    <col min="2" max="2" width="19.28515625" customWidth="1"/>
+    <col min="3" max="3" width="21.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -5729,7 +5729,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>36526</v>
       </c>
@@ -5740,7 +5740,7 @@
         <v>280443</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>36557</v>
       </c>
@@ -5751,7 +5751,7 @@
         <v>276823</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>36586</v>
       </c>
@@ -5762,7 +5762,7 @@
         <v>291681</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>36617</v>
       </c>
@@ -5773,7 +5773,7 @@
         <v>296155</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>36647</v>
       </c>
@@ -5784,7 +5784,7 @@
         <v>282343</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>36678</v>
       </c>
@@ -5795,7 +5795,7 @@
         <v>275888</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>36708</v>
       </c>
@@ -5806,7 +5806,7 @@
         <v>283867</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>36739</v>
       </c>
@@ -5817,7 +5817,7 @@
         <v>295251</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>36770</v>
       </c>
@@ -5828,7 +5828,7 @@
         <v>284468</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>36800</v>
       </c>
@@ -5839,7 +5839,7 @@
         <v>282529</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>36831</v>
       </c>
@@ -5850,7 +5850,7 @@
         <v>279618</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>36861</v>
       </c>
@@ -5861,7 +5861,7 @@
         <v>283932</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>36892</v>
       </c>
@@ -5872,7 +5872,7 @@
         <v>266629</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>36923</v>
       </c>
@@ -5883,7 +5883,7 @@
         <v>268091</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>36951</v>
       </c>
@@ -5894,7 +5894,7 @@
         <v>276803</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>36982</v>
       </c>
@@ -5905,7 +5905,7 @@
         <v>271578</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>37012</v>
       </c>
@@ -5916,7 +5916,7 @@
         <v>266005</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>37043</v>
       </c>
@@ -5927,7 +5927,7 @@
         <v>273520</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>37073</v>
       </c>
@@ -5938,7 +5938,7 @@
         <v>278574</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>37104</v>
       </c>
@@ -5961,13 +5961,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C606FF9A-90E0-4BFC-996A-18738DF4D853}">
   <dimension ref="A1:B37"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.1796875" customWidth="1"/>
-    <col min="2" max="2" width="9.26953125" customWidth="1"/>
+    <col min="1" max="1" width="17.140625" customWidth="1"/>
+    <col min="2" max="2" width="9.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -5975,7 +5975,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>41214</v>
       </c>
@@ -5983,7 +5983,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>41244</v>
       </c>
@@ -5991,7 +5991,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>41275</v>
       </c>
@@ -5999,7 +5999,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>41306</v>
       </c>
@@ -6007,7 +6007,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>41334</v>
       </c>
@@ -6015,7 +6015,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>41365</v>
       </c>
@@ -6023,7 +6023,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>41395</v>
       </c>
@@ -6031,7 +6031,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>41426</v>
       </c>
@@ -6039,7 +6039,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>41456</v>
       </c>
@@ -6047,7 +6047,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>41487</v>
       </c>
@@ -6055,7 +6055,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>41518</v>
       </c>
@@ -6063,7 +6063,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>41548</v>
       </c>
@@ -6071,7 +6071,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>41579</v>
       </c>
@@ -6079,7 +6079,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>41609</v>
       </c>
@@ -6087,7 +6087,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>41640</v>
       </c>
@@ -6095,7 +6095,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>41671</v>
       </c>
@@ -6103,7 +6103,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>41699</v>
       </c>
@@ -6111,7 +6111,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>41730</v>
       </c>
@@ -6119,7 +6119,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>41760</v>
       </c>
@@ -6127,7 +6127,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>41791</v>
       </c>
@@ -6135,7 +6135,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>41821</v>
       </c>
@@ -6143,7 +6143,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>41852</v>
       </c>
@@ -6151,7 +6151,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>41883</v>
       </c>
@@ -6159,7 +6159,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>41913</v>
       </c>
@@ -6167,7 +6167,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>41944</v>
       </c>
@@ -6175,7 +6175,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>41974</v>
       </c>
@@ -6183,7 +6183,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>42005</v>
       </c>
@@ -6191,7 +6191,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>42036</v>
       </c>
@@ -6199,7 +6199,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>42064</v>
       </c>
@@ -6207,7 +6207,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <v>42095</v>
       </c>
@@ -6215,7 +6215,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>42125</v>
       </c>
@@ -6223,7 +6223,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>42156</v>
       </c>
@@ -6231,7 +6231,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>42186</v>
       </c>
@@ -6239,7 +6239,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>42217</v>
       </c>
@@ -6247,7 +6247,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <v>42248</v>
       </c>
@@ -6255,7 +6255,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>42278</v>
       </c>
@@ -6275,9 +6275,9 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B3B220C-3A50-4B54-B01D-C649E0FAC685}">
   <dimension ref="A1:D37"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -6291,7 +6291,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>40725</v>
       </c>
@@ -6305,7 +6305,7 @@
         <v>8.6085909027762</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>40756</v>
       </c>
@@ -6319,7 +6319,7 @@
         <v>8.7906289699461198</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>40787</v>
       </c>
@@ -6333,7 +6333,7 @@
         <v>10.0857497060183</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>40817</v>
       </c>
@@ -6347,7 +6347,7 @@
         <v>10.3606397123789</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>40848</v>
       </c>
@@ -6361,7 +6361,7 @@
         <v>10.0489721368359</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>40878</v>
       </c>
@@ -6375,7 +6375,7 @@
         <v>8.8747874889107194</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>40909</v>
       </c>
@@ -6389,7 +6389,7 @@
         <v>9.4357162866803606</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>40940</v>
       </c>
@@ -6403,7 +6403,7 @@
         <v>9.4394819529891691</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>40969</v>
       </c>
@@ -6417,7 +6417,7 @@
         <v>11.1521380040711</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>41000</v>
       </c>
@@ -6431,7 +6431,7 @@
         <v>8.42396803326392</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>41030</v>
       </c>
@@ -6445,7 +6445,7 @@
         <v>8.9510993008145991</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>41061</v>
       </c>
@@ -6459,7 +6459,7 @@
         <v>10.731890179459301</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>41091</v>
       </c>
@@ -6473,7 +6473,7 @@
         <v>8.6952501061947096</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>41122</v>
       </c>
@@ -6487,7 +6487,7 @@
         <v>9.5560205906754394</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>41153</v>
       </c>
@@ -6501,7 +6501,7 @@
         <v>10.3161198440961</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>41183</v>
       </c>
@@ -6515,7 +6515,7 @@
         <v>9.9618027583798305</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>41214</v>
       </c>
@@ -6529,7 +6529,7 @@
         <v>9.6096906203913193</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>41244</v>
       </c>
@@ -6543,7 +6543,7 @@
         <v>9.2557775439294403</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>41275</v>
       </c>
@@ -6557,7 +6557,7 @@
         <v>8.4394797678994298</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>41306</v>
       </c>
@@ -6571,7 +6571,7 @@
         <v>9.4723407425707897</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>41334</v>
       </c>
@@ -6585,7 +6585,7 @@
         <v>9.5975243010892406</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>41365</v>
       </c>
@@ -6599,7 +6599,7 @@
         <v>8.7946563623140097</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>41395</v>
       </c>
@@ -6613,7 +6613,7 @@
         <v>9.9011828102910293</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>41426</v>
       </c>
@@ -6627,7 +6627,7 @@
         <v>10.6528050707009</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>41456</v>
       </c>
@@ -6641,7 +6641,7 @@
         <v>9.5917635967353405</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>41487</v>
       </c>
@@ -6655,7 +6655,7 @@
         <v>9.5528095261963397</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>41518</v>
       </c>
@@ -6669,7 +6669,7 @@
         <v>9.6754394391480396</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>41548</v>
       </c>
@@ -6683,7 +6683,7 @@
         <v>10.278452158237799</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>41579</v>
       </c>
@@ -6697,7 +6697,7 @@
         <v>8.5974976393376394</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <v>41609</v>
       </c>
@@ -6711,7 +6711,7 @@
         <v>9.8033121443617208</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>41640</v>
       </c>
@@ -6725,7 +6725,7 @@
         <v>7.8372733344789296</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>41671</v>
       </c>
@@ -6739,7 +6739,7 @@
         <v>8.8850727910671807</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>41699</v>
       </c>
@@ -6753,7 +6753,7 @@
         <v>9.3973397911971599</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>41730</v>
       </c>
@@ -6767,7 +6767,7 @@
         <v>9.7320308299828895</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <v>41760</v>
       </c>
@@ -6781,7 +6781,7 @@
         <v>8.5165372688354495</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>41791</v>
       </c>

</xml_diff>